<commit_message>
Verify Leslee B at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -559,7 +559,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
+    <row r="5" ht="110" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -575,12 +575,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Партнёрства (ведёт партнёров)</t>
+          <t>Партнёрские отношения, мероприятия, лидогенерация (вход и организатор звонка; не лицо, принимающее решение)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>США</t>
+          <t>США (Charleston, South Carolina, удалённо; в профиле также Boston)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -595,12 +595,12 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Самый логичный первый контакт: ведёт партнёрские отношения. Фамилия в Seamless сокращена.</t>
+          <t>Две роли с 03.2023: Sales and Marketing Specialist и Partner Manager &amp; Relationship Builder. Заголовок: Sales &amp; Event Leader | Relationship Building &amp; Lead Gen Expert. Подходит для реферальной схемы, совместных мероприятий и маркетинга; для условий сотрудничества и интеграции подключать Kevin Ebert или Ayaan Israni.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Kevin Ebert at RapDev and make him first
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -565,32 +565,32 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Leslee B</t>
+          <t>Kevin Ebert</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Partner Manager &amp; Relationship Builder</t>
+          <t>Head of Global Sales</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Партнёрские отношения, мероприятия, лидогенерация (вход и организатор звонка; не лицо, принимающее решение)</t>
+          <t>Продажи и партнёрские решения (что RapDev продаёт вместе с партнёром)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>США (Charleston, South Carolina, удалённо; в профиле также Boston)</t>
+          <t>Greater Boston, США</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>03.2023</t>
+          <t>09.2025 Head of Global Sales; Advisory Board Member RapDev с 06.2023</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/leslee-b-14092029</t>
+          <t>https://www.linkedin.com/in/kevin-ebert-8a68177</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -600,52 +600,52 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Две роли с 03.2023: Sales and Marketing Specialist и Partner Manager &amp; Relationship Builder. Заголовок: Sales &amp; Event Leader | Relationship Building &amp; Lead Gen Expert. Подходит для реферальной схемы, совместных мероприятий и маркетинга; для условий сотрудничества и интеграции подключать Kevin Ebert или Ayaan Israni.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="62" customHeight="1">
+          <t>Первым: руководитель продаж и бывший советник RapDev (с 2023), решает, что продавать вместе с партнёром. Ранее Airtable. 6 129 подписчиков. В активности личные посты (в письмо не использовать).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Kevin Ebert</t>
+          <t>Leslee B</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Head of Global Sales</t>
+          <t>Partner Manager &amp; Relationship Builder</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Продажи (решает, что продавать вместе с партнёром)</t>
+          <t>Партнёрские отношения, мероприятия, лидогенерация (вход и организатор звонка; не лицо, принимающее решение)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Massachusetts, США</t>
+          <t>США (Charleston, South Carolina, удалённо; в профиле также Boston)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>09.2025</t>
+          <t>03.2023</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/kevin-ebert-8a68177</t>
+          <t>https://www.linkedin.com/in/leslee-b-14092029</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Пришёл из Airtable (Head of Global Sales). Второй: коммерческое решение по совместным продажам и рефералам.</t>
+          <t>Две роли с 03.2023: Sales and Marketing Specialist и Partner Manager &amp; Relationship Builder. Заголовок: Sales &amp; Event Leader | Relationship Building &amp; Lead Gen Expert. Подходит для реферальной схемы, совместных мероприятий и маркетинга; для условий сотрудничества и интеграции подключать Kevin Ebert или Ayaan Israni. Вторая: писать через 3–5 дней после Kevin Ebert, для организации звонка и совместного маркетинга.</t>
         </is>
       </c>
     </row>
@@ -1099,6 +1099,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1179,7 +1180,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Leslee B → Kevin Ebert → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
+          <t>Kevin Ebert → Leslee B → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Ayaan Israni at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -649,7 +649,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="62" customHeight="1">
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -665,12 +665,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Первое лицо среди найденных</t>
+          <t>Первое лицо RapDev, решения о стратегическом партнёрстве</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>New York, США</t>
+          <t>Greater Boston, США (в Seamless был New York)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -685,12 +685,12 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Выходить после Leslee/Kevin или если они молчат. CEO/сооснователей в выдаче нет.</t>
+          <t>President с 2022 («Building RapDev.io»). До этого Head of Corporate Development в Cloud9 (Symphony), Strategic Market Infrastructure в J.P. Morgan, консалтинг. Бэкграунд в корпоративном развитии: подходит для стратегического партнёрства. Свежих постов нет, в сети не активен: шанс ответа на холодное письмо ниже. Ставить раньше, если партнёрство стратегическое.</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Verify Bob Kolosky at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -694,7 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="62" customHeight="1">
+    <row r="8" ht="130" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
@@ -705,17 +705,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager, ITOM Practice Lead</t>
+          <t>Sr. Engineering Manager, ITOM Practice Lead, ServiceNow CTA/ArchX</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Техническая практика ITOM (CMDB, мониторинг)</t>
+          <t>Технический руководитель практики ITOM: оценка технического соответствия и интеграций (не коммерческое решение)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>California, США</t>
+          <t>Murrieta, California, США (удалённо)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Для обсуждения технического соответствия и интеграций; практика ITOM рядом с CMDB.</t>
+          <t>17 лет на платформе ServiceNow, сертифицированный технический архитектор; ранее Stratascale, Cask, InSource. Подключать после интереса со стороны Kevin Ebert/Ayaan. Риск: ServiceNow для вас конкурент в CMDB (по документу); заходить через FinOps/облачные расходы, а не через CMDB, пока интеграция Cloudaware–ServiceNow не подтверждена.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Elias Kapetanopoulos at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -739,7 +739,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="62" customHeight="1">
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -750,17 +750,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Director of Engineering – ServiceNow</t>
+          <t>Director of ServiceNow Engineering (Director of Engineering – ServiceNow)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Инженерия ServiceNow</t>
+          <t>Руководитель инженерной команды ServiceNow: выполнение проектов, технический партнёр после коммерческого интереса</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Massachusetts, США</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Нужен, если партнёрство строится вокруг ServiceNow.</t>
+          <t>В RapDev 6 лет 3 мес.: от ServiceNow Engineer (08.2020) до директора (10.2024). В активности репосты про найм (Senior ServiceNow Engineer, Senior Project Manager): практика растёт. Не принимает коммерческих решений; подключать после интереса Kevin Ebert/Ayaan или если партнёрство строится вокруг ServiceNow. Интеграция Cloudaware–ServiceNow не подтверждена.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Connor Brackett and move him to third at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -559,7 +559,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
+    <row r="5" ht="130" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -604,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="130" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -649,38 +649,38 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="110" customHeight="1">
+    <row r="7" ht="130" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ayaan Israni</t>
+          <t>Connor Brackett</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Director of Sales, Americas</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Первое лицо RapDev, решения о стратегическом партнёрстве</t>
+          <t>Продажи по Америке; инсайдер (сотрудник №3), чемпион внутри компании, работает с клиентами напрямую</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Greater Boston, США (в Seamless был New York)</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>01.2022</t>
+          <t>11.2019 (7 лет)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ayaanisrani</t>
+          <t>https://www.linkedin.com/in/connorbrackett</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>President с 2022 («Building RapDev.io»). До этого Head of Corporate Development в Cloud9 (Symphony), Strategic Market Infrastructure в J.P. Morgan, консалтинг. Бэкграунд в корпоративном развитии: подходит для стратегического партнёрства. Свежих постов нет, в сети не активен: шанс ответа на холодное письмо ниже. Ставить раньше, если партнёрство стратегическое.</t>
+          <t>Сотрудник номер 3 в RapDev, строит компанию с 2019 года; ранее AppNeta (продажи). 1 670 подписчиков, активен в LinkedIn, репостит события и вебинары. Доступнее Ayaan для холодного захода. RapDev описывает себя как ServiceNow Elite partner на стыке ServiceNow и DevOps, cloud-native и контейнеры.</t>
         </is>
       </c>
     </row>
@@ -700,32 +700,32 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Bob Kolosky</t>
+          <t>Ayaan Israni</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sr. Engineering Manager, ITOM Practice Lead, ServiceNow CTA/ArchX</t>
+          <t>President</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Технический руководитель практики ITOM: оценка технического соответствия и интеграций (не коммерческое решение)</t>
+          <t>Первое лицо RapDev, решения о стратегическом партнёрстве</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Murrieta, California, США (удалённо)</t>
+          <t>Greater Boston, США (в Seamless был New York)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>12.2022</t>
+          <t>01.2022</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bkolosky</t>
+          <t>https://www.linkedin.com/in/ayaanisrani</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -735,42 +735,42 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>17 лет на платформе ServiceNow, сертифицированный технический архитектор; ранее Stratascale, Cask, InSource. Подключать после интереса со стороны Kevin Ebert/Ayaan. Риск: ServiceNow для вас конкурент в CMDB (по документу); заходить через FinOps/облачные расходы, а не через CMDB, пока интеграция Cloudaware–ServiceNow не подтверждена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="120" customHeight="1">
+          <t>President с 2022 («Building RapDev.io»). До этого Head of Corporate Development в Cloud9 (Symphony), Strategic Market Infrastructure в J.P. Morgan, консалтинг. Бэкграунд в корпоративном развитии: подходит для стратегического партнёрства. Свежих постов нет, в сети не активен: шанс ответа на холодное письмо ниже. Ставить раньше, если партнёрство стратегическое.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="130" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Elias Kapetanopoulos</t>
+          <t>Bob Kolosky</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Director of ServiceNow Engineering (Director of Engineering – ServiceNow)</t>
+          <t>Sr. Engineering Manager, ITOM Practice Lead, ServiceNow CTA/ArchX</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Руководитель инженерной команды ServiceNow: выполнение проектов, технический партнёр после коммерческого интереса</t>
+          <t>Технический руководитель практики ITOM: оценка технического соответствия и интеграций (не коммерческое решение)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Boston, Massachusetts, США</t>
+          <t>Murrieta, California, США (удалённо)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10.2024 в должности (в RapDev с 08.2020)</t>
+          <t>12.2022</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/elias-kapetanopoulos</t>
+          <t>https://www.linkedin.com/in/bkolosky</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -780,52 +780,52 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>В RapDev 6 лет 3 мес.: от ServiceNow Engineer (08.2020) до директора (10.2024). В активности репосты про найм (Senior ServiceNow Engineer, Senior Project Manager): практика растёт. Не принимает коммерческих решений; подключать после интереса Kevin Ebert/Ayaan или если партнёрство строится вокруг ServiceNow. Интеграция Cloudaware–ServiceNow не подтверждена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="62" customHeight="1">
+          <t>17 лет на платформе ServiceNow, сертифицированный технический архитектор; ранее Stratascale, Cask, InSource. Подключать после интереса со стороны Kevin Ebert/Ayaan. Риск: ServiceNow для вас конкурент в CMDB (по документу); заходить через FinOps/облачные расходы, а не через CMDB, пока интеграция Cloudaware–ServiceNow не подтверждена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="130" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Connor Brackett</t>
+          <t>Elias Kapetanopoulos</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Director of Sales</t>
+          <t>Director of ServiceNow Engineering (Director of Engineering – ServiceNow)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Продажи (директор)</t>
+          <t>Руководитель инженерной команды ServiceNow: выполнение проектов, технический партнёр после коммерческого интереса</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Boston, США</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>11.2019</t>
+          <t>10.2024 в должности (в RapDev с 08.2020)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/connorbrackett</t>
+          <t>https://www.linkedin.com/in/elias-kapetanopoulos</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>В RapDev с 2019 года. Полезен для конкретных сделок после первого разговора.</t>
+          <t>В RapDev 6 лет 3 мес.: от ServiceNow Engineer (08.2020) до директора (10.2024). В активности репосты про найм (Senior ServiceNow Engineer, Senior Project Manager): практика растёт. Не принимает коммерческих решений; подключать после интереса Kevin Ebert/Ayaan или если партнёрство строится вокруг ServiceNow. Интеграция Cloudaware–ServiceNow не подтверждена.</t>
         </is>
       </c>
     </row>
@@ -1099,6 +1099,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1179,7 +1180,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Kevin Ebert → Leslee B → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
+          <t>Kevin Ebert → Leslee B → Connor Brackett → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Jesse Eddy and add RapDev founder Tameem Hourani
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -745,42 +745,42 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Bob Kolosky</t>
+          <t>Tameem Hourani</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Sr. Engineering Manager, ITOM Practice Lead, ServiceNow CTA/ArchX</t>
+          <t>Founder @ RapDev.io (в Seamless: Principal)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Технический руководитель практики ITOM: оценка технического соответствия и интеграций (не коммерческое решение)</t>
+          <t>Основатель RapDev: стратегическое решение о партнёрстве</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Murrieta, California, США (удалённо)</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>12.2022</t>
+          <t>07.2019 в Seamless (основана в 2017)</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bkolosky</t>
+          <t>https://www.linkedin.com/in/tameem-hourani</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Да (по скриншоту профиля)</t>
+          <t>Нет (подпись «Founder @ RapDev.io» видна в посте, репостнутом Jesse Eddy; сам профиль не открывали)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>17 лет на платформе ServiceNow, сертифицированный технический архитектор; ранее Stratascale, Cask, InSource. Подключать после интереса со стороны Kevin Ebert/Ayaan. Риск: ServiceNow для вас конкурент в CMDB (по документу); заходить через FinOps/облачные расходы, а не через CMDB, пока интеграция Cloudaware–ServiceNow не подтверждена.</t>
+          <t>В Seamless значится «Principal» с 2019 года, ранее Wayfair (Director of Production Operations). Основатель по подписи в посте. Поднять в списке после проверки профиля.</t>
         </is>
       </c>
     </row>
@@ -790,32 +790,32 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Elias Kapetanopoulos</t>
+          <t>Bob Kolosky</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Director of ServiceNow Engineering (Director of Engineering – ServiceNow)</t>
+          <t>Sr. Engineering Manager, ITOM Practice Lead, ServiceNow CTA/ArchX</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Руководитель инженерной команды ServiceNow: выполнение проектов, технический партнёр после коммерческого интереса</t>
+          <t>Технический руководитель практики ITOM: оценка технического соответствия и интеграций (не коммерческое решение)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Boston, Massachusetts, США</t>
+          <t>Murrieta, California, США (удалённо)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>10.2024 в должности (в RapDev с 08.2020)</t>
+          <t>12.2022</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/elias-kapetanopoulos</t>
+          <t>https://www.linkedin.com/in/bkolosky</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -825,97 +825,97 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>В RapDev 6 лет 3 мес.: от ServiceNow Engineer (08.2020) до директора (10.2024). В активности репосты про найм (Senior ServiceNow Engineer, Senior Project Manager): практика растёт. Не принимает коммерческих решений; подключать после интереса Kevin Ebert/Ayaan или если партнёрство строится вокруг ServiceNow. Интеграция Cloudaware–ServiceNow не подтверждена.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1">
+          <t>17 лет на платформе ServiceNow, сертифицированный технический архитектор; ранее Stratascale, Cask, InSource. Подключать после интереса со стороны Kevin Ebert/Ayaan. Риск: ServiceNow для вас конкурент в CMDB (по документу); заходить через FinOps/облачные расходы, а не через CMDB, пока интеграция Cloudaware–ServiceNow не подтверждена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="130" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Jesse Eddy</t>
+          <t>Elias Kapetanopoulos</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Regional Sales Director</t>
+          <t>Director of ServiceNow Engineering (Director of Engineering – ServiceNow)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Региональные продажи</t>
+          <t>Руководитель инженерной команды ServiceNow: выполнение проектов, технический партнёр после коммерческого интереса</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Massachusetts, США</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>10.2024</t>
+          <t>10.2024 в должности (в RapDev с 08.2020)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jesseeddy</t>
+          <t>https://www.linkedin.com/in/elias-kapetanopoulos</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Для конкретных сделок и клиентов.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="62" customHeight="1">
+          <t>В RapDev 6 лет 3 мес.: от ServiceNow Engineer (08.2020) до директора (10.2024). В активности репосты про найм (Senior ServiceNow Engineer, Senior Project Manager): практика растёт. Не принимает коммерческих решений; подключать после интереса Kevin Ebert/Ayaan или если партнёрство строится вокруг ServiceNow. Интеграция Cloudaware–ServiceNow не подтверждена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="130" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Ryan Henrich</t>
+          <t>Jesse Eddy</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Director of Sales, Security</t>
+          <t>Regional Sales Director</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Продажи по безопасности</t>
+          <t>Региональные продажи Datadog и ServiceNow; кандидат в чемпионы для совместных продаж на уровне полевых продаж</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Santa Monica, США</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>07.2024</t>
+          <t>10.2024 в должности (в RapDev 6 лет)</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ryanhenrich</t>
+          <t>https://www.linkedin.com/in/jesseeddy</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Актуален, если партнёрство затрагивает безопасность и compliance.</t>
+          <t>Ранее Principal Enterprise Account Executive и Enterprise AE в RapDev, до этого Cloudreach (AWS-консалтинг) и Datadog (3 года 7 мес., Senior AE, Team Lead). Знает облачную экосистему и клиентов Datadog. Для конкретных сделок после первого разговора с Kevin/Connor.</t>
         </is>
       </c>
     </row>
@@ -925,32 +925,32 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Jared Kennedy</t>
+          <t>Ryan Henrich</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Datadog Sales Lead, APJ</t>
+          <t>Director of Sales, Security</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Продажи Datadog, Азиатско-Тихоокеанский регион</t>
+          <t>Продажи по безопасности</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Австралия</t>
+          <t>Santa Monica, США</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>07.2026</t>
+          <t>07.2024</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jared-kennedy-96761560</t>
+          <t>https://www.linkedin.com/in/ryanhenrich</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Региональная роль, APAC. Низкий приоритет для США.</t>
+          <t>Актуален, если партнёрство затрагивает безопасность и compliance.</t>
         </is>
       </c>
     </row>
@@ -970,32 +970,32 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Jessy Lamontagne</t>
+          <t>Jared Kennedy</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Sales Operations Lead</t>
+          <t>Datadog Sales Lead, APJ</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Операции продаж</t>
+          <t>Продажи Datadog, Азиатско-Тихоокеанский регион</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Nashua, New Hampshire, США</t>
+          <t>Австралия</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>10.2025</t>
+          <t>07.2026</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jessy-lamontagne-079b97103</t>
+          <t>https://www.linkedin.com/in/jared-kennedy-96761560</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Для процессов, не для решений о партнёрстве.</t>
+          <t>Региональная роль, APAC. Низкий приоритет для США.</t>
         </is>
       </c>
     </row>
@@ -1015,47 +1015,95 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>Jessy Lamontagne</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Sales Operations Lead</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Операции продаж</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Nashua, New Hampshire, США</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>10.2025</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jessy-lamontagne-079b97103</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Для процессов, не для решений о партнёрстве.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="62" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>Eyob Tesfaye</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Technical Partner</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Непонятно (по названию — технический партнёр)</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Эфиопия</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>04.2024</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/eyob-tesfaye-34b9a9319</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Роль не ясна, возможно, консультант или подрядчик. Низкий приоритет.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Зелёным выделены первые пять: основной список для партнёрского разговора.</t>
         </is>
@@ -1074,6 +1122,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1099,7 +1148,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1132,7 +1180,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>68 по запросу «ServiceNow/CTO/VP/Alliances…», просмотрены первые 10; CEO или сооснователей не найдено, только President</t>
+          <t>68 по запросу «ServiceNow/CTO/VP/Alliances…», просмотрены первые 10; CEO или сооснователей не найдено, только President. Основатель Tameem Hourani в Seamless записан как «Principal» и найден только по имени</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1228,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Kevin Ebert → Leslee B → Connor Brackett → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
+          <t>Kevin Ebert → Leslee B → Connor Brackett → Ayaan Israni → Tameem Hourani (основатель; проверить профиль); техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify founder Tameem Hourani and move him to third at RapDev
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/RapDev_contacts.xlsx
+++ b/RapDev_contacts.xlsx
@@ -559,7 +559,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="130" customHeight="1">
+    <row r="5" ht="135" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -604,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="130" customHeight="1">
+    <row r="6" ht="135" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -649,23 +649,23 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="130" customHeight="1">
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Connor Brackett</t>
+          <t>Tameem Hourani</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Director of Sales, Americas</t>
+          <t>Founder @ RapDev.io (в опыте: Principal с 07.2019; в Seamless: Principal)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Продажи по Америке; инсайдер (сотрудник №3), чемпион внутри компании, работает с клиентами напрямую</t>
+          <t>Основатель RapDev: стратегическое решение о партнёрстве; доступен через общих знакомых</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>11.2019 (7 лет)</t>
+          <t>07.2019 (7 лет 4 мес.); компания основана в 2017</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/connorbrackett</t>
+          <t>https://www.linkedin.com/in/tameem-hourani</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -690,42 +690,42 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Сотрудник номер 3 в RapDev, строит компанию с 2019 года; ранее AppNeta (продажи). 1 670 подписчиков, активен в LinkedIn, репостит события и вебинары. Доступнее Ayaan для холодного захода. RapDev описывает себя как ServiceNow Elite partner на стыке ServiceNow и DevOps, cloud-native и контейнеры.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="130" customHeight="1">
+          <t>Во втором круге (2nd), общие знакомые: Bobby, Vaibhav и ещё один: просить представить через «Get introduced». 7 205 подписчиков, активно пишет (культура, команда доставки, бонус за продление клиентов). RapDev на 246-м месте в рейтинге Forbes лучших работодателей. Лучший путь: знакомство через общих знакомых, а не холодное письмо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="135" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Ayaan Israni</t>
+          <t>Connor Brackett</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Director of Sales, Americas</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Первое лицо RapDev, решения о стратегическом партнёрстве</t>
+          <t>Продажи по Америке; инсайдер (сотрудник №3), чемпион внутри компании, работает с клиентами напрямую</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Greater Boston, США (в Seamless был New York)</t>
+          <t>Boston, Massachusetts, США</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>01.2022</t>
+          <t>11.2019 (7 лет)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ayaanisrani</t>
+          <t>https://www.linkedin.com/in/connorbrackett</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -735,56 +735,56 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>President с 2022 («Building RapDev.io»). До этого Head of Corporate Development в Cloud9 (Symphony), Strategic Market Infrastructure в J.P. Morgan, консалтинг. Бэкграунд в корпоративном развитии: подходит для стратегического партнёрства. Свежих постов нет, в сети не активен: шанс ответа на холодное письмо ниже. Ставить раньше, если партнёрство стратегическое.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="130" customHeight="1">
+          <t>Сотрудник номер 3 в RapDev, строит компанию с 2019 года; ранее AppNeta (продажи). 1 670 подписчиков, активен в LinkedIn, репостит события и вебинары. Доступнее Ayaan для холодного захода. RapDev описывает себя как ServiceNow Elite partner на стыке ServiceNow и DevOps, cloud-native и контейнеры.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="135" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Tameem Hourani</t>
+          <t>Ayaan Israni</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Founder @ RapDev.io (в Seamless: Principal)</t>
+          <t>President</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Основатель RapDev: стратегическое решение о партнёрстве</t>
+          <t>Первое лицо RapDev, решения о стратегическом партнёрстве</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Boston, Massachusetts, США</t>
+          <t>Greater Boston, США (в Seamless был New York)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>07.2019 в Seamless (основана в 2017)</t>
+          <t>01.2022</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/tameem-hourani</t>
+          <t>https://www.linkedin.com/in/ayaanisrani</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Нет (подпись «Founder @ RapDev.io» видна в посте, репостнутом Jesse Eddy; сам профиль не открывали)</t>
+          <t>Да (по скриншоту профиля)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>В Seamless значится «Principal» с 2019 года, ранее Wayfair (Director of Production Operations). Основатель по подписи в посте. Поднять в списке после проверки профиля.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="130" customHeight="1">
+          <t>President с 2022 («Building RapDev.io»). До этого Head of Corporate Development в Cloud9 (Symphony), Strategic Market Infrastructure в J.P. Morgan, консалтинг. Бэкграунд в корпоративном развитии: подходит для стратегического партнёрства. Свежих постов нет, в сети не активен: шанс ответа на холодное письмо ниже. Ставить раньше, если партнёрство стратегическое.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="135" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
@@ -829,7 +829,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="130" customHeight="1">
+    <row r="11" ht="135" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
@@ -874,7 +874,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="130" customHeight="1">
+    <row r="12" ht="135" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
@@ -1148,6 +1148,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1228,7 +1229,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Kevin Ebert → Leslee B → Connor Brackett → Ayaan Israni → Tameem Hourani (основатель; проверить профиль); техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
+          <t>Kevin Ebert → Leslee B → Tameem Hourani (основатель; лучше через общих знакомых: он во втором круге) → Connor Brackett → Ayaan Israni; техническим руководителям (Bob Kolosky, Elias Kapetanopoulos) — после первого разговора или если партнёрство техническое. Не писать всем в один день</t>
         </is>
       </c>
     </row>

</xml_diff>